<commit_message>
feat: load real home test products into Excel database
</commit_message>
<xml_diff>
--- a/datos/inventario.xlsx
+++ b/datos/inventario.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,16 +449,16 @@
         <v>ART-001</v>
       </c>
       <c r="C2" t="str">
-        <v>Motor Trifasico 5HP Siemens</v>
+        <v>Calculadora Cientifica Casio fx-350MS</v>
       </c>
       <c r="D2" t="str">
-        <v>Motores</v>
+        <v>Electronica y Oficina</v>
       </c>
       <c r="E2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F2">
-        <v>450</v>
+        <v>25</v>
       </c>
       <c r="G2" t="str">
         <v>USD</v>
@@ -467,19 +467,19 @@
         <v>A</v>
       </c>
       <c r="I2" t="str">
-        <v>12</v>
+        <v>01</v>
       </c>
       <c r="J2" t="str">
         <v>2</v>
       </c>
       <c r="K2" t="str">
-        <v>Motor electrico trifasico de alto rendimiento con rotor de jaula de ardilla.</v>
+        <v>Calculadora cientifica de 2 lineas con 240 funciones, display S-V.P.A.M. ideal para medicion y calculo en taller.</v>
       </c>
       <c r="L2" t="str">
         <v>Disponible</v>
       </c>
       <c r="M2" t="str">
-        <v>Siemens Argentina</v>
+        <v>Casio Argentina</v>
       </c>
     </row>
     <row r="3">
@@ -490,22 +490,22 @@
         <v>ART-002</v>
       </c>
       <c r="C3" t="str">
-        <v>Sensor Fotoelectrico Omron E3Z</v>
+        <v>Cargador Rapido Samsung USB-C</v>
       </c>
       <c r="D3" t="str">
-        <v>Sensores</v>
+        <v>Accesorios y Alimentacion</v>
       </c>
       <c r="E3">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>85.5</v>
+        <v>19.5</v>
       </c>
       <c r="G3" t="str">
         <v>USD</v>
       </c>
       <c r="H3" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="I3" t="str">
         <v>04</v>
@@ -514,13 +514,13 @@
         <v>1</v>
       </c>
       <c r="K3" t="str">
-        <v>Sensor optico difuso infrarrojo con alcance de deteccion de hasta 1 metro.</v>
+        <v>Adaptador de corriente de carga rapida con cable reforzado USB tipo C para dispositivos de planta.</v>
       </c>
       <c r="L3" t="str">
         <v>Disponible</v>
       </c>
       <c r="M3" t="str">
-        <v>Omron Automation</v>
+        <v>Samsung</v>
       </c>
     </row>
     <row r="4">
@@ -531,37 +531,37 @@
         <v>ART-003</v>
       </c>
       <c r="C4" t="str">
-        <v>PLC Schneider Modicon M221</v>
+        <v>Joystick Sony DualShock 4 PS4 Negro</v>
       </c>
       <c r="D4" t="str">
-        <v>Automatizacion</v>
+        <v>Control y Telemando</v>
       </c>
       <c r="E4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F4">
-        <v>320</v>
+        <v>65</v>
       </c>
       <c r="G4" t="str">
         <v>USD</v>
       </c>
       <c r="H4" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="I4" t="str">
-        <v>03</v>
+        <v>02</v>
       </c>
       <c r="J4" t="str">
         <v>3</v>
       </c>
       <c r="K4" t="str">
-        <v>Controlador logico programable de 24 E/S para aplicaciones de control discreto.</v>
+        <v>Controlador inalambrico con panel tactil y sensores de movimiento de 6 ejes, apto para teleoperacion y simuladores.</v>
       </c>
       <c r="L4" t="str">
-        <v>Stock Bajo</v>
+        <v>Stock Critico</v>
       </c>
       <c r="M4" t="str">
-        <v>Schneider Electric</v>
+        <v>Sony PlayStation</v>
       </c>
     </row>
     <row r="5">
@@ -572,131 +572,49 @@
         <v>ART-004</v>
       </c>
       <c r="C5" t="str">
-        <v>Valvula Solenoide Neumatica Festo 5/2</v>
+        <v>Auriculares Gamer Headset con Microfono</v>
       </c>
       <c r="D5" t="str">
-        <v>Neumatica</v>
+        <v>Audio y Comunicacion</v>
       </c>
       <c r="E5">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F5">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="G5" t="str">
         <v>USD</v>
       </c>
       <c r="H5" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="I5" t="str">
-        <v>08</v>
+        <v>05</v>
       </c>
       <c r="J5" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="str">
-        <v>Electrovalvula biestable de actuacion neumatica rapida a 24VDC.</v>
+        <v>Auriculares circumaurales acolchados con cancelacion pasiva de ruido y microfono flexible para comunicaciones de sala.</v>
       </c>
       <c r="L5" t="str">
         <v>Disponible</v>
       </c>
       <c r="M5" t="str">
-        <v>Festo</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>ART-005</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Rodamiento Rigido SKF 6205-2RSH</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Mecanica</v>
-      </c>
-      <c r="E6">
-        <v>120</v>
-      </c>
-      <c r="F6">
-        <v>14.2</v>
-      </c>
-      <c r="G6" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H6" t="str">
-        <v>D</v>
-      </c>
-      <c r="I6" t="str">
-        <v>15</v>
-      </c>
-      <c r="J6" t="str">
-        <v>4</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Rodamiento de una hilera de bolas con obturacion en ambos lados de caucho.</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Disponible</v>
-      </c>
-      <c r="M6" t="str">
-        <v>SKF</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>ART-006</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Variador de Frecuencia WEG CFW500</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Accionamientos</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>290</v>
-      </c>
-      <c r="G7" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H7" t="str">
-        <v>B</v>
-      </c>
-      <c r="I7" t="str">
-        <v>07</v>
-      </c>
-      <c r="J7" t="str">
-        <v>2</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Convertidor de frecuencia para control de velocidad de motores trifasicos de induccion.</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Stock Critico</v>
-      </c>
-      <c r="M7" t="str">
-        <v>WEG</v>
+        <v>Gaming Audio Pro</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -714,10 +632,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Motores</v>
+        <v>Electronica y Oficina</v>
       </c>
       <c r="C2" t="str">
-        <v>Motores electricos y actuadores principales</v>
+        <v>Equipos de computo y oficina tecnica</v>
       </c>
     </row>
     <row r="3">
@@ -725,10 +643,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Sensores</v>
+        <v>Accesorios y Alimentacion</v>
       </c>
       <c r="C3" t="str">
-        <v>Dispositivos de medicion y deteccion</v>
+        <v>Cargadores, fuentes y conectividad</v>
       </c>
     </row>
     <row r="4">
@@ -736,10 +654,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Automatizacion</v>
+        <v>Control y Telemando</v>
       </c>
       <c r="C4" t="str">
-        <v>Controladores logicos programables y modulos I/O</v>
+        <v>Controladores, periféricos y simuladores</v>
       </c>
     </row>
     <row r="5">
@@ -747,37 +665,15 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Neumatica</v>
+        <v>Audio y Comunicacion</v>
       </c>
       <c r="C5" t="str">
-        <v>Valvulas, cilindros y actuadores por aire</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Mecanica</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Rodamientos, poleas, engranajes y acoples</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Accionamientos</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Variadores de velocidad y arrancadores suaves</v>
+        <v>Headsets y sistemas de diadema para comunicación</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: non-intrusive bottom drawer AR card and live bidirectional Excel stock editing
</commit_message>
<xml_diff>
--- a/datos/inventario.xlsx
+++ b/datos/inventario.xlsx
@@ -537,7 +537,7 @@
         <v>Control y Telemando</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4">
         <v>65</v>
@@ -558,7 +558,7 @@
         <v>Controlador inalambrico con panel tactil y sensores de movimiento de 6 ejes, apto para teleoperacion y simuladores.</v>
       </c>
       <c r="L4" t="str">
-        <v>Stock Critico</v>
+        <v>Stock Bajo</v>
       </c>
       <c r="M4" t="str">
         <v>Sony PlayStation</v>

</xml_diff>